<commit_message>
data: refresh leaderboard (2026-10-19)
</commit_message>
<xml_diff>
--- a/public/downloads/RolingConfigurational2017.xlsx
+++ b/public/downloads/RolingConfigurational2017.xlsx
@@ -11,13 +11,14 @@
     <sheet name="MLIP_Data_shifted" sheetId="2" r:id="rId2"/>
     <sheet name="anomaly" sheetId="3" r:id="rId3"/>
     <sheet name="anomaly_shifted" sheetId="4" r:id="rId4"/>
+    <sheet name="Coverage" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="76">
   <si>
     <t>MLIP_name</t>
   </si>
@@ -70,39 +71,72 @@
     <t>energy anomaly</t>
   </si>
   <si>
+    <t>Allegro-OAM-L</t>
+  </si>
+  <si>
     <t>AlphaNet-v1-OMA</t>
   </si>
   <si>
-    <t>CHGNetv0.3.0</t>
+    <t>CHGNet-v0.3.0</t>
   </si>
   <si>
     <t>DPA-3.1-3M-FT</t>
   </si>
   <si>
+    <t>DPA-4.0.1-pro-MPtrj</t>
+  </si>
+  <si>
     <t>Eqnorm-MPtrj</t>
   </si>
   <si>
+    <t>EquFlash</t>
+  </si>
+  <si>
+    <t>EquFlashV2</t>
+  </si>
+  <si>
     <t>eSEN-30M-OAM</t>
   </si>
   <si>
     <t>GRACE-2L-OAM</t>
   </si>
   <si>
+    <t>MACE-MH-1-OC20</t>
+  </si>
+  <si>
+    <t>MACE-MH-1-OMAT</t>
+  </si>
+  <si>
     <t>MACE-MPA-0</t>
   </si>
   <si>
-    <t>MATLANTISv8</t>
-  </si>
-  <si>
-    <t>MatterSim_v1_5M</t>
+    <t>MatterSim-v1-5M</t>
+  </si>
+  <si>
+    <t>NequIP-OAM-L</t>
+  </si>
+  <si>
+    <t>NequIP-OAM-XL</t>
+  </si>
+  <si>
+    <t>Nequix-MP-1</t>
   </si>
   <si>
     <t>ORB-v3</t>
   </si>
   <si>
+    <t>PET-OAM-XL</t>
+  </si>
+  <si>
     <t>SevenNet-MF-OMPA</t>
   </si>
   <si>
+    <t>SevenNet-Omni</t>
+  </si>
+  <si>
+    <t>TACE-OAM-L</t>
+  </si>
+  <si>
     <t>Num_normal</t>
   </si>
   <si>
@@ -137,6 +171,81 @@
   </si>
   <si>
     <t>slab_move</t>
+  </si>
+  <si>
+    <t>Num_input</t>
+  </si>
+  <si>
+    <t>Num_succeeded</t>
+  </si>
+  <si>
+    <t>Num_failed</t>
+  </si>
+  <si>
+    <t>Num_not_run</t>
+  </si>
+  <si>
+    <t>Coverage_pct</t>
+  </si>
+  <si>
+    <t>Failed_by_stage</t>
+  </si>
+  <si>
+    <t>catbench_version</t>
+  </si>
+  <si>
+    <t>dispersion</t>
+  </si>
+  <si>
+    <t>device</t>
+  </si>
+  <si>
+    <t>input_md5</t>
+  </si>
+  <si>
+    <t>EqV3-OMatMPtrjSalex</t>
+  </si>
+  <si>
+    <t>MatRIS-10M-OAM</t>
+  </si>
+  <si>
+    <t>UMA-m-1p1-OC20</t>
+  </si>
+  <si>
+    <t>UMA-m-1p1-OMAT</t>
+  </si>
+  <si>
+    <t>UMA-s-1p1-OC20</t>
+  </si>
+  <si>
+    <t>UMA-s-1p1-OMAT</t>
+  </si>
+  <si>
+    <t>UMA-s-1p2-OC20</t>
+  </si>
+  <si>
+    <t>UMA-s-1p2-OC22</t>
+  </si>
+  <si>
+    <t>UMA-s-1p2-OMAT</t>
+  </si>
+  <si>
+    <t>unknown: 104</t>
+  </si>
+  <si>
+    <t>1.1.4</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>NVIDIA L40S</t>
+  </si>
+  <si>
+    <t>unknown</t>
+  </si>
+  <si>
+    <t>Num_succeeded counts every computed reaction, including any later excluded by energy_cutoff, so it can exceed Num_total in MLIP_Data.</t>
   </si>
 </sst>
 </file>
@@ -173,7 +282,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -181,11 +290,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -201,6 +325,9 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -496,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -604,31 +731,31 @@
         <v>0</v>
       </c>
       <c r="H3" s="4">
-        <v>0.4895208264221995</v>
+        <v>0.507388473764984</v>
       </c>
       <c r="I3" s="4">
-        <v>0.4895208264221995</v>
+        <v>0.507388473764984</v>
       </c>
       <c r="J3" s="4">
-        <v>0.4881485673340282</v>
+        <v>0.5055625663110329</v>
       </c>
       <c r="K3" s="4">
-        <v>86.07993197278911</v>
+        <v>91.00536368393512</v>
       </c>
       <c r="L3" s="4">
-        <v>90.96551798313544</v>
+        <v>93.7751677852349</v>
       </c>
       <c r="M3" s="5">
         <v>104</v>
       </c>
       <c r="N3" s="5">
-        <v>200952.0864486694</v>
+        <v>29868.53837966919</v>
       </c>
       <c r="O3" s="4">
-        <v>30.84926104523633</v>
+        <v>7.469001845378642</v>
       </c>
       <c r="P3" s="5">
-        <v>6514</v>
+        <v>3999</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="25" customHeight="1">
@@ -654,31 +781,31 @@
         <v>0</v>
       </c>
       <c r="H4" s="4">
-        <v>0.2922057904781124</v>
+        <v>0.4903489825266542</v>
       </c>
       <c r="I4" s="4">
-        <v>0.2922057904781124</v>
+        <v>0.4903489825266542</v>
       </c>
       <c r="J4" s="4">
-        <v>0.2941959380774859</v>
+        <v>0.4881502546039727</v>
       </c>
       <c r="K4" s="4">
-        <v>80.64887493458922</v>
+        <v>89.07018576661433</v>
       </c>
       <c r="L4" s="4">
-        <v>86.32184649802096</v>
+        <v>92.81707107210461</v>
       </c>
       <c r="M4" s="5">
         <v>104</v>
       </c>
       <c r="N4" s="5">
-        <v>405786.9956493378</v>
+        <v>91564.697265625</v>
       </c>
       <c r="O4" s="4">
-        <v>44.30472711533331</v>
+        <v>19.6998057800398</v>
       </c>
       <c r="P4" s="5">
-        <v>9159</v>
+        <v>4648</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="25" customHeight="1">
@@ -704,31 +831,31 @@
         <v>0</v>
       </c>
       <c r="H5" s="4">
-        <v>0.5191341806633484</v>
+        <v>0.2925306999817557</v>
       </c>
       <c r="I5" s="4">
-        <v>0.5191341806633484</v>
+        <v>0.2925306999817557</v>
       </c>
       <c r="J5" s="4">
-        <v>0.5145763945837949</v>
+        <v>0.2941966716731139</v>
       </c>
       <c r="K5" s="4">
-        <v>85.13343799058082</v>
+        <v>82.32240973312398</v>
       </c>
       <c r="L5" s="4">
-        <v>90.6692049561177</v>
+        <v>88.34720788160386</v>
       </c>
       <c r="M5" s="5">
         <v>104</v>
       </c>
       <c r="N5" s="5">
-        <v>1016029.210090637</v>
+        <v>196273.4065055847</v>
       </c>
       <c r="O5" s="4">
-        <v>160.0550110413732</v>
+        <v>27.93529839248288</v>
       </c>
       <c r="P5" s="5">
-        <v>6348</v>
+        <v>7026</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="25" customHeight="1">
@@ -754,31 +881,31 @@
         <v>0</v>
       </c>
       <c r="H6" s="4">
-        <v>0.3750562585122688</v>
+        <v>0.5194893265573394</v>
       </c>
       <c r="I6" s="4">
-        <v>0.3750562585122688</v>
+        <v>0.5194893265573394</v>
       </c>
       <c r="J6" s="4">
-        <v>0.3520749955995359</v>
+        <v>0.5145761680574886</v>
       </c>
       <c r="K6" s="4">
-        <v>84.63108320251176</v>
+        <v>88.01020408163265</v>
       </c>
       <c r="L6" s="4">
-        <v>89.35209086215797</v>
+        <v>92.60325245224574</v>
       </c>
       <c r="M6" s="5">
         <v>104</v>
       </c>
       <c r="N6" s="5">
-        <v>633747.8663921356</v>
+        <v>388136.1019611359</v>
       </c>
       <c r="O6" s="4">
-        <v>84.73697906032031</v>
+        <v>85.45488814644119</v>
       </c>
       <c r="P6" s="5">
-        <v>7479</v>
+        <v>4542</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="25" customHeight="1">
@@ -786,13 +913,13 @@
         <v>21</v>
       </c>
       <c r="B7" s="3">
-        <v>35.57692307692308</v>
+        <v>100</v>
       </c>
       <c r="C7" s="3">
         <v>0</v>
       </c>
       <c r="D7" s="3">
-        <v>64.42307692307693</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3">
         <v>0</v>
@@ -801,34 +928,34 @@
         <v>0</v>
       </c>
       <c r="G7" s="3">
-        <v>64.42307692307693</v>
+        <v>0</v>
       </c>
       <c r="H7" s="4">
-        <v>2.819678386845216</v>
+        <v>0.5299612308462167</v>
       </c>
       <c r="I7" s="4">
-        <v>1.480429705142253</v>
+        <v>0.5299612308462167</v>
       </c>
       <c r="J7" s="4">
-        <v>2.822534274625039</v>
+        <v>0.5255289735052465</v>
       </c>
       <c r="K7" s="4">
-        <v>88.9046964939822</v>
+        <v>87.58993982208267</v>
       </c>
       <c r="L7" s="4">
-        <v>92.65767509895028</v>
+        <v>91.31410256410255</v>
       </c>
       <c r="M7" s="5">
         <v>104</v>
       </c>
       <c r="N7" s="5">
-        <v>796950.3824710846</v>
+        <v>410550.7462024689</v>
       </c>
       <c r="O7" s="4">
-        <v>156.1423163148677</v>
+        <v>79.28751375095962</v>
       </c>
       <c r="P7" s="5">
-        <v>5104</v>
+        <v>5178</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="25" customHeight="1">
@@ -836,13 +963,13 @@
         <v>22</v>
       </c>
       <c r="B8" s="3">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C8" s="3">
         <v>0</v>
       </c>
       <c r="D8" s="3">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E8" s="3">
         <v>0</v>
@@ -851,34 +978,34 @@
         <v>0</v>
       </c>
       <c r="G8" s="3">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H8" s="4">
-        <v>1.399493235316091</v>
+        <v>0.3727272757922605</v>
       </c>
       <c r="I8" s="4">
-        <v>1.156295698267128</v>
+        <v>0.3727272757922605</v>
       </c>
       <c r="J8" s="4">
-        <v>1.39655183745886</v>
+        <v>0.3520755091164756</v>
       </c>
       <c r="K8" s="4">
-        <v>86.36087127158555</v>
+        <v>86.43543956043956</v>
       </c>
       <c r="L8" s="4">
-        <v>91.02123128549302</v>
+        <v>91.06124161073825</v>
       </c>
       <c r="M8" s="5">
         <v>104</v>
       </c>
       <c r="N8" s="5">
-        <v>75619.4908618927</v>
+        <v>295400.2401828766</v>
       </c>
       <c r="O8" s="4">
-        <v>12.41087983947033</v>
+        <v>51.72478378267844</v>
       </c>
       <c r="P8" s="5">
-        <v>6093</v>
+        <v>5711</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="25" customHeight="1">
@@ -886,49 +1013,49 @@
         <v>23</v>
       </c>
       <c r="B9" s="3">
-        <v>98.07692307692307</v>
+        <v>100</v>
       </c>
       <c r="C9" s="3">
         <v>0</v>
       </c>
       <c r="D9" s="3">
-        <v>1.923076923076923</v>
+        <v>0</v>
       </c>
       <c r="E9" s="3">
         <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>1.923076923076923</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3">
         <v>0</v>
       </c>
       <c r="H9" s="4">
-        <v>0.3625311883592286</v>
+        <v>0.4774830937099513</v>
       </c>
       <c r="I9" s="4">
-        <v>0.3664552748070886</v>
+        <v>0.4774830937099513</v>
       </c>
       <c r="J9" s="4">
-        <v>0.359130904405522</v>
+        <v>0.4765842189869571</v>
       </c>
       <c r="K9" s="4">
-        <v>86.20290423861852</v>
+        <v>90.61813186813185</v>
       </c>
       <c r="L9" s="4">
-        <v>89.95622526243322</v>
+        <v>93.7013853037343</v>
       </c>
       <c r="M9" s="5">
         <v>104</v>
       </c>
       <c r="N9" s="5">
-        <v>217739.2194271088</v>
+        <v>255651.2842178345</v>
       </c>
       <c r="O9" s="4">
-        <v>28.574700712219</v>
+        <v>61.52858825940661</v>
       </c>
       <c r="P9" s="5">
-        <v>7620</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="25" customHeight="1">
@@ -936,13 +1063,13 @@
         <v>24</v>
       </c>
       <c r="B10" s="3">
-        <v>96.15384615384616</v>
+        <v>100</v>
       </c>
       <c r="C10" s="3">
         <v>0</v>
       </c>
       <c r="D10" s="3">
-        <v>3.846153846153846</v>
+        <v>0</v>
       </c>
       <c r="E10" s="3">
         <v>0</v>
@@ -951,34 +1078,34 @@
         <v>0</v>
       </c>
       <c r="G10" s="3">
-        <v>3.846153846153846</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>0.6471977043606103</v>
+        <v>0.6475186725935627</v>
       </c>
       <c r="I10" s="4">
-        <v>0.5854266032842842</v>
+        <v>0.6475186725935627</v>
       </c>
       <c r="J10" s="4">
-        <v>0.6440337911499274</v>
+        <v>0.6442896047177739</v>
       </c>
       <c r="K10" s="4">
-        <v>84.19250392464679</v>
+        <v>89.943746729461</v>
       </c>
       <c r="L10" s="4">
-        <v>89.80801497160557</v>
+        <v>93.6923507141628</v>
       </c>
       <c r="M10" s="5">
         <v>104</v>
       </c>
       <c r="N10" s="5">
-        <v>585141.1719322205</v>
+        <v>567468.0647850037</v>
       </c>
       <c r="O10" s="4">
-        <v>88.0971351900362</v>
+        <v>147.1267992701591</v>
       </c>
       <c r="P10" s="5">
-        <v>6642</v>
+        <v>3857</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="25" customHeight="1">
@@ -986,13 +1113,13 @@
         <v>25</v>
       </c>
       <c r="B11" s="3">
-        <v>100</v>
+        <v>35.57692307692308</v>
       </c>
       <c r="C11" s="3">
         <v>0</v>
       </c>
       <c r="D11" s="3">
-        <v>0</v>
+        <v>64.42307692307693</v>
       </c>
       <c r="E11" s="3">
         <v>0</v>
@@ -1001,34 +1128,34 @@
         <v>0</v>
       </c>
       <c r="G11" s="3">
-        <v>0</v>
+        <v>64.42307692307693</v>
       </c>
       <c r="H11" s="4">
-        <v>0.9176693558978978</v>
+        <v>2.819698870210642</v>
       </c>
       <c r="I11" s="4">
-        <v>0.9176693558978978</v>
+        <v>1.48069264217253</v>
       </c>
       <c r="J11" s="4">
-        <v>0.918936275547462</v>
+        <v>2.822534510751131</v>
       </c>
       <c r="K11" s="4">
-        <v>86.07110151753011</v>
+        <v>90.76497906855049</v>
       </c>
       <c r="L11" s="4">
-        <v>90.10185424195491</v>
+        <v>93.99059972466013</v>
       </c>
       <c r="M11" s="5">
         <v>104</v>
       </c>
       <c r="N11" s="5">
-        <v>263616.1639690399</v>
+        <v>313611.2062931061</v>
       </c>
       <c r="O11" s="4">
-        <v>38.45043231753791</v>
+        <v>85.96798418122425</v>
       </c>
       <c r="P11" s="5">
-        <v>6856</v>
+        <v>3648</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="25" customHeight="1">
@@ -1036,13 +1163,13 @@
         <v>26</v>
       </c>
       <c r="B12" s="3">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C12" s="3">
         <v>0</v>
       </c>
       <c r="D12" s="3">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E12" s="3">
         <v>0</v>
@@ -1051,34 +1178,34 @@
         <v>0</v>
       </c>
       <c r="G12" s="3">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H12" s="4">
-        <v>0.3916222588216177</v>
+        <v>1.399676815241166</v>
       </c>
       <c r="I12" s="4">
-        <v>0.3916222588216177</v>
+        <v>1.156448170432014</v>
       </c>
       <c r="J12" s="4">
-        <v>0.3946323239401593</v>
+        <v>1.396551837458862</v>
       </c>
       <c r="K12" s="4">
-        <v>81.09399529042385</v>
+        <v>88.82751177394034</v>
       </c>
       <c r="L12" s="4">
-        <v>87.67983135432802</v>
+        <v>92.73102736189985</v>
       </c>
       <c r="M12" s="5">
         <v>104</v>
       </c>
       <c r="N12" s="5">
-        <v>131943.7901973724</v>
+        <v>28272.83668518066</v>
       </c>
       <c r="O12" s="4">
-        <v>17.60424152066343</v>
+        <v>6.618173381362515</v>
       </c>
       <c r="P12" s="5">
-        <v>7495</v>
+        <v>4272</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="25" customHeight="1">
@@ -1104,31 +1231,581 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>0.5372718526480805</v>
+        <v>0.2043416563215944</v>
       </c>
       <c r="I13" s="4">
-        <v>0.5372718526480805</v>
+        <v>0.2043416563215944</v>
       </c>
       <c r="J13" s="4">
-        <v>0.5339133785035117</v>
+        <v>0.2032706687010133</v>
       </c>
       <c r="K13" s="4">
-        <v>87.70408163265306</v>
+        <v>84.11793563579278</v>
       </c>
       <c r="L13" s="4">
-        <v>91.93200395801065</v>
+        <v>90.75019359834796</v>
       </c>
       <c r="M13" s="5">
         <v>104</v>
       </c>
       <c r="N13" s="5">
-        <v>409228.9431095123</v>
+        <v>143733.3271503448</v>
       </c>
       <c r="O13" s="4">
-        <v>72.40427160465541</v>
+        <v>29.7215316688058</v>
       </c>
       <c r="P13" s="5">
-        <v>5652</v>
+        <v>4836</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="25" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="3">
+        <v>100</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0.2043416563215985</v>
+      </c>
+      <c r="I14" s="4">
+        <v>0.2043416563215985</v>
+      </c>
+      <c r="J14" s="4">
+        <v>0.2032706687010144</v>
+      </c>
+      <c r="K14" s="4">
+        <v>84.11793563579278</v>
+      </c>
+      <c r="L14" s="4">
+        <v>90.75019359834796</v>
+      </c>
+      <c r="M14" s="5">
+        <v>104</v>
+      </c>
+      <c r="N14" s="5">
+        <v>143946.0480213165</v>
+      </c>
+      <c r="O14" s="4">
+        <v>29.76551861482972</v>
+      </c>
+      <c r="P14" s="5">
+        <v>4836</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="3">
+        <v>100</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0.519273576186738</v>
+      </c>
+      <c r="I15" s="4">
+        <v>0.519273576186738</v>
+      </c>
+      <c r="J15" s="4">
+        <v>0.5185478999969719</v>
+      </c>
+      <c r="K15" s="4">
+        <v>91.65423861852433</v>
+      </c>
+      <c r="L15" s="4">
+        <v>93.57931078988125</v>
+      </c>
+      <c r="M15" s="5">
+        <v>104</v>
+      </c>
+      <c r="N15" s="5">
+        <v>121592.4944877625</v>
+      </c>
+      <c r="O15" s="4">
+        <v>26.93078504712347</v>
+      </c>
+      <c r="P15" s="5">
+        <v>4515</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="25" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="3">
+        <v>100</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4">
+        <v>0.9173489224738284</v>
+      </c>
+      <c r="I16" s="4">
+        <v>0.9173489224738284</v>
+      </c>
+      <c r="J16" s="4">
+        <v>0.9189364967723936</v>
+      </c>
+      <c r="K16" s="4">
+        <v>88.00791470434328</v>
+      </c>
+      <c r="L16" s="4">
+        <v>91.62267681982443</v>
+      </c>
+      <c r="M16" s="5">
+        <v>104</v>
+      </c>
+      <c r="N16" s="5">
+        <v>115730.6454181671</v>
+      </c>
+      <c r="O16" s="4">
+        <v>22.06915435129045</v>
+      </c>
+      <c r="P16" s="5">
+        <v>5244</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="25" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="3">
+        <v>100</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0.5035449697274971</v>
+      </c>
+      <c r="I17" s="4">
+        <v>0.5035449697274971</v>
+      </c>
+      <c r="J17" s="4">
+        <v>0.5003795078822189</v>
+      </c>
+      <c r="K17" s="4">
+        <v>89.75176609105179</v>
+      </c>
+      <c r="L17" s="4">
+        <v>93.63943383238686</v>
+      </c>
+      <c r="M17" s="5">
+        <v>104</v>
+      </c>
+      <c r="N17" s="5">
+        <v>16254.96554374695</v>
+      </c>
+      <c r="O17" s="4">
+        <v>4.107901325182448</v>
+      </c>
+      <c r="P17" s="5">
+        <v>3957</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="25" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="3">
+        <v>100</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0.5070908271694919</v>
+      </c>
+      <c r="I18" s="4">
+        <v>0.5070908271694919</v>
+      </c>
+      <c r="J18" s="4">
+        <v>0.5044726137899816</v>
+      </c>
+      <c r="K18" s="4">
+        <v>90.14782836211408</v>
+      </c>
+      <c r="L18" s="4">
+        <v>93.75677594217863</v>
+      </c>
+      <c r="M18" s="5">
+        <v>104</v>
+      </c>
+      <c r="N18" s="5">
+        <v>22964.25485610962</v>
+      </c>
+      <c r="O18" s="4">
+        <v>6.027363479293864</v>
+      </c>
+      <c r="P18" s="5">
+        <v>3810</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="25" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="3">
+        <v>100</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0.3272499347165126</v>
+      </c>
+      <c r="I19" s="4">
+        <v>0.3272499347165126</v>
+      </c>
+      <c r="J19" s="4">
+        <v>0.311410400735226</v>
+      </c>
+      <c r="K19" s="4">
+        <v>87.56377551020405</v>
+      </c>
+      <c r="L19" s="4">
+        <v>91.12512906556525</v>
+      </c>
+      <c r="M19" s="5">
+        <v>104</v>
+      </c>
+      <c r="N19" s="5">
+        <v>128687.6938343048</v>
+      </c>
+      <c r="O19" s="4">
+        <v>20.71264990090211</v>
+      </c>
+      <c r="P19" s="5">
+        <v>6213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="3">
+        <v>100</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0</v>
+      </c>
+      <c r="F20" s="3">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0.391714872977167</v>
+      </c>
+      <c r="I20" s="4">
+        <v>0.391714872977167</v>
+      </c>
+      <c r="J20" s="4">
+        <v>0.3946868278028337</v>
+      </c>
+      <c r="K20" s="4">
+        <v>84.60295656724229</v>
+      </c>
+      <c r="L20" s="4">
+        <v>90.18843572534847</v>
+      </c>
+      <c r="M20" s="5">
+        <v>104</v>
+      </c>
+      <c r="N20" s="5">
+        <v>54562.0813369751</v>
+      </c>
+      <c r="O20" s="4">
+        <v>10.04086885111798</v>
+      </c>
+      <c r="P20" s="5">
+        <v>5434</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="25" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="3">
+        <v>25</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>75</v>
+      </c>
+      <c r="E21" s="3">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <v>75</v>
+      </c>
+      <c r="H21" s="4">
+        <v>3.446118776643454</v>
+      </c>
+      <c r="I21" s="4">
+        <v>1.531679212913941</v>
+      </c>
+      <c r="J21" s="4">
+        <v>3.450093984632486</v>
+      </c>
+      <c r="K21" s="4">
+        <v>87.66287284144425</v>
+      </c>
+      <c r="L21" s="4">
+        <v>92.14969454482878</v>
+      </c>
+      <c r="M21" s="5">
+        <v>104</v>
+      </c>
+      <c r="N21" s="5">
+        <v>233471.5230464935</v>
+      </c>
+      <c r="O21" s="4">
+        <v>55.19421348616868</v>
+      </c>
+      <c r="P21" s="5">
+        <v>4230</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="25" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="3">
+        <v>100</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4">
+        <v>0.5371911023958886</v>
+      </c>
+      <c r="I22" s="4">
+        <v>0.5371911023958886</v>
+      </c>
+      <c r="J22" s="4">
+        <v>0.5339120032982699</v>
+      </c>
+      <c r="K22" s="4">
+        <v>89.7723704866562</v>
+      </c>
+      <c r="L22" s="4">
+        <v>93.48025296850801</v>
+      </c>
+      <c r="M22" s="5">
+        <v>104</v>
+      </c>
+      <c r="N22" s="5">
+        <v>99616.95075035095</v>
+      </c>
+      <c r="O22" s="4">
+        <v>25.28990879673799</v>
+      </c>
+      <c r="P22" s="5">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="25" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="3">
+        <v>100</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4">
+        <v>0.5205318818585746</v>
+      </c>
+      <c r="I23" s="4">
+        <v>0.5205318818585746</v>
+      </c>
+      <c r="J23" s="4">
+        <v>0.5175491553946698</v>
+      </c>
+      <c r="K23" s="4">
+        <v>89.22782574568288</v>
+      </c>
+      <c r="L23" s="4">
+        <v>93.19469540526588</v>
+      </c>
+      <c r="M23" s="5">
+        <v>104</v>
+      </c>
+      <c r="N23" s="5">
+        <v>101589.7951126099</v>
+      </c>
+      <c r="O23" s="4">
+        <v>25.00979692580253</v>
+      </c>
+      <c r="P23" s="5">
+        <v>4062</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="25" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="3">
+        <v>100</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4">
+        <v>0.5104261905815108</v>
+      </c>
+      <c r="I24" s="4">
+        <v>0.5104261905815108</v>
+      </c>
+      <c r="J24" s="4">
+        <v>0.5072674045876712</v>
+      </c>
+      <c r="K24" s="4">
+        <v>89.70434327577185</v>
+      </c>
+      <c r="L24" s="4">
+        <v>93.45895715023229</v>
+      </c>
+      <c r="M24" s="5">
+        <v>104</v>
+      </c>
+      <c r="N24" s="5">
+        <v>571849.1594791412</v>
+      </c>
+      <c r="O24" s="4">
+        <v>143.2846804006869</v>
+      </c>
+      <c r="P24" s="5">
+        <v>3991</v>
       </c>
     </row>
   </sheetData>
@@ -1153,7 +1830,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -1261,31 +1938,31 @@
         <v>0</v>
       </c>
       <c r="H3" s="4">
-        <v>0.1005989086363357</v>
+        <v>0.09727370120366564</v>
       </c>
       <c r="I3" s="4">
-        <v>0.1005989086363357</v>
+        <v>0.09727370120366564</v>
       </c>
       <c r="J3" s="4">
-        <v>0.1049615737171289</v>
+        <v>0.1016269506308224</v>
       </c>
       <c r="K3" s="4">
-        <v>86.07993197278911</v>
+        <v>91.00536368393512</v>
       </c>
       <c r="L3" s="4">
-        <v>90.96551798313544</v>
+        <v>93.7751677852349</v>
       </c>
       <c r="M3" s="5">
         <v>104</v>
       </c>
       <c r="N3" s="5">
-        <v>200952.0864486694</v>
+        <v>29868.53837966919</v>
       </c>
       <c r="O3" s="4">
-        <v>30.84926104523633</v>
+        <v>7.469001845378642</v>
       </c>
       <c r="P3" s="5">
-        <v>6514</v>
+        <v>3999</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="25" customHeight="1">
@@ -1311,31 +1988,31 @@
         <v>0</v>
       </c>
       <c r="H4" s="4">
-        <v>0.1112572368332909</v>
+        <v>0.1003780963523062</v>
       </c>
       <c r="I4" s="4">
-        <v>0.1112572368332909</v>
+        <v>0.1003780963523062</v>
       </c>
       <c r="J4" s="4">
-        <v>0.1156466066650382</v>
+        <v>0.1050284372495357</v>
       </c>
       <c r="K4" s="4">
-        <v>80.64887493458922</v>
+        <v>89.07018576661433</v>
       </c>
       <c r="L4" s="4">
-        <v>86.32184649802096</v>
+        <v>92.81707107210461</v>
       </c>
       <c r="M4" s="5">
         <v>104</v>
       </c>
       <c r="N4" s="5">
-        <v>405786.9956493378</v>
+        <v>91564.697265625</v>
       </c>
       <c r="O4" s="4">
-        <v>44.30472711533331</v>
+        <v>19.6998057800398</v>
       </c>
       <c r="P4" s="5">
-        <v>9159</v>
+        <v>4648</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="25" customHeight="1">
@@ -1361,31 +2038,31 @@
         <v>0</v>
       </c>
       <c r="H5" s="4">
-        <v>0.05774538022553489</v>
+        <v>0.1106547916596583</v>
       </c>
       <c r="I5" s="4">
-        <v>0.05774538022553489</v>
+        <v>0.1106547916596583</v>
       </c>
       <c r="J5" s="4">
-        <v>0.06130283441841488</v>
+        <v>0.1156797739051471</v>
       </c>
       <c r="K5" s="4">
-        <v>85.13343799058082</v>
+        <v>82.32240973312398</v>
       </c>
       <c r="L5" s="4">
-        <v>90.6692049561177</v>
+        <v>88.34720788160386</v>
       </c>
       <c r="M5" s="5">
         <v>104</v>
       </c>
       <c r="N5" s="5">
-        <v>1016029.210090637</v>
+        <v>196273.4065055847</v>
       </c>
       <c r="O5" s="4">
-        <v>160.0550110413732</v>
+        <v>27.93529839248288</v>
       </c>
       <c r="P5" s="5">
-        <v>6348</v>
+        <v>7026</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="25" customHeight="1">
@@ -1411,31 +2088,31 @@
         <v>0</v>
       </c>
       <c r="H6" s="4">
-        <v>0.1357814276975879</v>
+        <v>0.05777400249058035</v>
       </c>
       <c r="I6" s="4">
-        <v>0.1357814276975879</v>
+        <v>0.05777400249058035</v>
       </c>
       <c r="J6" s="4">
-        <v>0.1162895868535269</v>
+        <v>0.06128974611243262</v>
       </c>
       <c r="K6" s="4">
-        <v>84.63108320251176</v>
+        <v>88.01020408163265</v>
       </c>
       <c r="L6" s="4">
-        <v>89.35209086215797</v>
+        <v>92.60325245224574</v>
       </c>
       <c r="M6" s="5">
         <v>104</v>
       </c>
       <c r="N6" s="5">
-        <v>633747.8663921356</v>
+        <v>388136.1019611359</v>
       </c>
       <c r="O6" s="4">
-        <v>84.73697906032031</v>
+        <v>85.45488814644119</v>
       </c>
       <c r="P6" s="5">
-        <v>7479</v>
+        <v>4542</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="25" customHeight="1">
@@ -1461,31 +2138,31 @@
         <v>0</v>
       </c>
       <c r="H7" s="4">
-        <v>0.04687695756587142</v>
+        <v>0.08196134572686345</v>
       </c>
       <c r="I7" s="4">
-        <v>0.04687695756587142</v>
+        <v>0.08196134572686345</v>
       </c>
       <c r="J7" s="4">
-        <v>0.04856542516489483</v>
+        <v>0.08428702652603456</v>
       </c>
       <c r="K7" s="4">
-        <v>88.9046964939822</v>
+        <v>87.58993982208267</v>
       </c>
       <c r="L7" s="4">
-        <v>92.65767509895028</v>
+        <v>91.31410256410255</v>
       </c>
       <c r="M7" s="5">
         <v>104</v>
       </c>
       <c r="N7" s="5">
-        <v>796950.3824710846</v>
+        <v>410550.7462024689</v>
       </c>
       <c r="O7" s="4">
-        <v>156.1423163148677</v>
+        <v>79.28751375095962</v>
       </c>
       <c r="P7" s="5">
-        <v>5104</v>
+        <v>5178</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="25" customHeight="1">
@@ -1511,31 +2188,31 @@
         <v>0</v>
       </c>
       <c r="H8" s="4">
-        <v>0.09690767885427592</v>
+        <v>0.1348645739616587</v>
       </c>
       <c r="I8" s="4">
-        <v>0.09690767885427592</v>
+        <v>0.1348645739616587</v>
       </c>
       <c r="J8" s="4">
-        <v>0.1023403012096705</v>
+        <v>0.115032674864236</v>
       </c>
       <c r="K8" s="4">
-        <v>86.36087127158555</v>
+        <v>86.43543956043956</v>
       </c>
       <c r="L8" s="4">
-        <v>91.02123128549302</v>
+        <v>91.06124161073825</v>
       </c>
       <c r="M8" s="5">
         <v>104</v>
       </c>
       <c r="N8" s="5">
-        <v>75619.4908618927</v>
+        <v>295400.2401828766</v>
       </c>
       <c r="O8" s="4">
-        <v>12.41087983947033</v>
+        <v>51.72478378267844</v>
       </c>
       <c r="P8" s="5">
-        <v>6093</v>
+        <v>5711</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="25" customHeight="1">
@@ -1543,49 +2220,49 @@
         <v>23</v>
       </c>
       <c r="B9" s="3">
-        <v>98.07692307692307</v>
+        <v>100</v>
       </c>
       <c r="C9" s="3">
         <v>0</v>
       </c>
       <c r="D9" s="3">
-        <v>1.923076923076923</v>
+        <v>0</v>
       </c>
       <c r="E9" s="3">
         <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>1.923076923076923</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3">
         <v>0</v>
       </c>
       <c r="H9" s="4">
-        <v>0.1070501417518825</v>
+        <v>0.06699404906723558</v>
       </c>
       <c r="I9" s="4">
-        <v>0.1052336260459115</v>
+        <v>0.06699404906723558</v>
       </c>
       <c r="J9" s="4">
-        <v>0.1009769846691031</v>
+        <v>0.0691030607243735</v>
       </c>
       <c r="K9" s="4">
-        <v>86.20290423861852</v>
+        <v>90.61813186813185</v>
       </c>
       <c r="L9" s="4">
-        <v>89.95622526243322</v>
+        <v>93.7013853037343</v>
       </c>
       <c r="M9" s="5">
         <v>104</v>
       </c>
       <c r="N9" s="5">
-        <v>217739.2194271088</v>
+        <v>255651.2842178345</v>
       </c>
       <c r="O9" s="4">
-        <v>28.574700712219</v>
+        <v>61.52858825940661</v>
       </c>
       <c r="P9" s="5">
-        <v>7620</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="25" customHeight="1">
@@ -1611,31 +2288,31 @@
         <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>0.07922659438918471</v>
+        <v>0.04019789757801383</v>
       </c>
       <c r="I10" s="4">
-        <v>0.07922659438918471</v>
+        <v>0.04019789757801383</v>
       </c>
       <c r="J10" s="4">
-        <v>0.07682239533936074</v>
+        <v>0.04062815028179535</v>
       </c>
       <c r="K10" s="4">
-        <v>84.19250392464679</v>
+        <v>89.943746729461</v>
       </c>
       <c r="L10" s="4">
-        <v>89.80801497160557</v>
+        <v>93.6923507141628</v>
       </c>
       <c r="M10" s="5">
         <v>104</v>
       </c>
       <c r="N10" s="5">
-        <v>585141.1719322205</v>
+        <v>567468.0647850037</v>
       </c>
       <c r="O10" s="4">
-        <v>88.0971351900362</v>
+        <v>147.1267992701591</v>
       </c>
       <c r="P10" s="5">
-        <v>6642</v>
+        <v>3857</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="25" customHeight="1">
@@ -1661,31 +2338,31 @@
         <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>0.1287227703516346</v>
+        <v>0.04684908093200724</v>
       </c>
       <c r="I11" s="4">
-        <v>0.1287227703516346</v>
+        <v>0.04684908093200724</v>
       </c>
       <c r="J11" s="4">
-        <v>0.1356971553415685</v>
+        <v>0.04859917056378306</v>
       </c>
       <c r="K11" s="4">
-        <v>86.07110151753011</v>
+        <v>90.76497906855049</v>
       </c>
       <c r="L11" s="4">
-        <v>90.10185424195491</v>
+        <v>93.99059972466013</v>
       </c>
       <c r="M11" s="5">
         <v>104</v>
       </c>
       <c r="N11" s="5">
-        <v>263616.1639690399</v>
+        <v>313611.2062931061</v>
       </c>
       <c r="O11" s="4">
-        <v>38.45043231753791</v>
+        <v>85.96798418122425</v>
       </c>
       <c r="P11" s="5">
-        <v>6856</v>
+        <v>3648</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="25" customHeight="1">
@@ -1711,31 +2388,31 @@
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>0.08542840203686528</v>
+        <v>0.0969903997739147</v>
       </c>
       <c r="I12" s="4">
-        <v>0.08542840203686528</v>
+        <v>0.0969903997739147</v>
       </c>
       <c r="J12" s="4">
-        <v>0.0842464974244021</v>
+        <v>0.102252093312594</v>
       </c>
       <c r="K12" s="4">
-        <v>81.09399529042385</v>
+        <v>88.82751177394034</v>
       </c>
       <c r="L12" s="4">
-        <v>87.67983135432802</v>
+        <v>92.73102736189985</v>
       </c>
       <c r="M12" s="5">
         <v>104</v>
       </c>
       <c r="N12" s="5">
-        <v>131943.7901973724</v>
+        <v>28272.83668518066</v>
       </c>
       <c r="O12" s="4">
-        <v>17.60424152066343</v>
+        <v>6.618173381362515</v>
       </c>
       <c r="P12" s="5">
-        <v>7495</v>
+        <v>4272</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="25" customHeight="1">
@@ -1761,31 +2438,581 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>0.06349033074889873</v>
+        <v>0.07318217147505159</v>
       </c>
       <c r="I13" s="4">
-        <v>0.06349033074889873</v>
+        <v>0.07318217147505159</v>
       </c>
       <c r="J13" s="4">
-        <v>0.06519168237916163</v>
+        <v>0.0753292060938333</v>
       </c>
       <c r="K13" s="4">
-        <v>87.70408163265306</v>
+        <v>84.11793563579278</v>
       </c>
       <c r="L13" s="4">
-        <v>91.93200395801065</v>
+        <v>90.75019359834796</v>
       </c>
       <c r="M13" s="5">
         <v>104</v>
       </c>
       <c r="N13" s="5">
-        <v>409228.9431095123</v>
+        <v>143733.3271503448</v>
       </c>
       <c r="O13" s="4">
-        <v>72.40427160465541</v>
+        <v>29.7215316688058</v>
       </c>
       <c r="P13" s="5">
-        <v>5652</v>
+        <v>4836</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="25" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="3">
+        <v>100</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0.07318217147504859</v>
+      </c>
+      <c r="I14" s="4">
+        <v>0.07318217147504859</v>
+      </c>
+      <c r="J14" s="4">
+        <v>0.07532920609382729</v>
+      </c>
+      <c r="K14" s="4">
+        <v>84.11793563579278</v>
+      </c>
+      <c r="L14" s="4">
+        <v>90.75019359834796</v>
+      </c>
+      <c r="M14" s="5">
+        <v>104</v>
+      </c>
+      <c r="N14" s="5">
+        <v>143946.0480213165</v>
+      </c>
+      <c r="O14" s="4">
+        <v>29.76551861482972</v>
+      </c>
+      <c r="P14" s="5">
+        <v>4836</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="3">
+        <v>100</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0.1214049771264056</v>
+      </c>
+      <c r="I15" s="4">
+        <v>0.1214049771264056</v>
+      </c>
+      <c r="J15" s="4">
+        <v>0.13152812783065</v>
+      </c>
+      <c r="K15" s="4">
+        <v>91.65423861852433</v>
+      </c>
+      <c r="L15" s="4">
+        <v>93.57931078988125</v>
+      </c>
+      <c r="M15" s="5">
+        <v>104</v>
+      </c>
+      <c r="N15" s="5">
+        <v>121592.4944877625</v>
+      </c>
+      <c r="O15" s="4">
+        <v>26.93078504712347</v>
+      </c>
+      <c r="P15" s="5">
+        <v>4515</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="25" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="3">
+        <v>100</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4">
+        <v>0.1285474409965414</v>
+      </c>
+      <c r="I16" s="4">
+        <v>0.1285474409965414</v>
+      </c>
+      <c r="J16" s="4">
+        <v>0.1356969352628801</v>
+      </c>
+      <c r="K16" s="4">
+        <v>88.00791470434328</v>
+      </c>
+      <c r="L16" s="4">
+        <v>91.62267681982443</v>
+      </c>
+      <c r="M16" s="5">
+        <v>104</v>
+      </c>
+      <c r="N16" s="5">
+        <v>115730.6454181671</v>
+      </c>
+      <c r="O16" s="4">
+        <v>22.06915435129045</v>
+      </c>
+      <c r="P16" s="5">
+        <v>5244</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="25" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="3">
+        <v>100</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0.06833560226908675</v>
+      </c>
+      <c r="I17" s="4">
+        <v>0.06833560226908675</v>
+      </c>
+      <c r="J17" s="4">
+        <v>0.06991820334485467</v>
+      </c>
+      <c r="K17" s="4">
+        <v>89.75176609105179</v>
+      </c>
+      <c r="L17" s="4">
+        <v>93.63943383238686</v>
+      </c>
+      <c r="M17" s="5">
+        <v>104</v>
+      </c>
+      <c r="N17" s="5">
+        <v>16254.96554374695</v>
+      </c>
+      <c r="O17" s="4">
+        <v>4.107901325182448</v>
+      </c>
+      <c r="P17" s="5">
+        <v>3957</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="25" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="3">
+        <v>100</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0.05584574983429139</v>
+      </c>
+      <c r="I18" s="4">
+        <v>0.05584574983429139</v>
+      </c>
+      <c r="J18" s="4">
+        <v>0.0579961604398157</v>
+      </c>
+      <c r="K18" s="4">
+        <v>90.14782836211408</v>
+      </c>
+      <c r="L18" s="4">
+        <v>93.75677594217863</v>
+      </c>
+      <c r="M18" s="5">
+        <v>104</v>
+      </c>
+      <c r="N18" s="5">
+        <v>22964.25485610962</v>
+      </c>
+      <c r="O18" s="4">
+        <v>6.027363479293864</v>
+      </c>
+      <c r="P18" s="5">
+        <v>3810</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="25" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="3">
+        <v>100</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0.1727321391747836</v>
+      </c>
+      <c r="I19" s="4">
+        <v>0.1727321391747836</v>
+      </c>
+      <c r="J19" s="4">
+        <v>0.1612614233979064</v>
+      </c>
+      <c r="K19" s="4">
+        <v>87.56377551020405</v>
+      </c>
+      <c r="L19" s="4">
+        <v>91.12512906556525</v>
+      </c>
+      <c r="M19" s="5">
+        <v>104</v>
+      </c>
+      <c r="N19" s="5">
+        <v>128687.6938343048</v>
+      </c>
+      <c r="O19" s="4">
+        <v>20.71264990090211</v>
+      </c>
+      <c r="P19" s="5">
+        <v>6213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="3">
+        <v>100</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0</v>
+      </c>
+      <c r="F20" s="3">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0.08520476389602843</v>
+      </c>
+      <c r="I20" s="4">
+        <v>0.08520476389602843</v>
+      </c>
+      <c r="J20" s="4">
+        <v>0.0843314157901255</v>
+      </c>
+      <c r="K20" s="4">
+        <v>84.60295656724229</v>
+      </c>
+      <c r="L20" s="4">
+        <v>90.18843572534847</v>
+      </c>
+      <c r="M20" s="5">
+        <v>104</v>
+      </c>
+      <c r="N20" s="5">
+        <v>54562.0813369751</v>
+      </c>
+      <c r="O20" s="4">
+        <v>10.04086885111798</v>
+      </c>
+      <c r="P20" s="5">
+        <v>5434</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="25" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="3">
+        <v>100</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4">
+        <v>0.06502861451846004</v>
+      </c>
+      <c r="I21" s="4">
+        <v>0.06502861451846004</v>
+      </c>
+      <c r="J21" s="4">
+        <v>0.06650457063864933</v>
+      </c>
+      <c r="K21" s="4">
+        <v>87.66287284144425</v>
+      </c>
+      <c r="L21" s="4">
+        <v>92.14969454482878</v>
+      </c>
+      <c r="M21" s="5">
+        <v>104</v>
+      </c>
+      <c r="N21" s="5">
+        <v>233471.5230464935</v>
+      </c>
+      <c r="O21" s="4">
+        <v>55.19421348616868</v>
+      </c>
+      <c r="P21" s="5">
+        <v>4230</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="25" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="3">
+        <v>100</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4">
+        <v>0.06337301378887469</v>
+      </c>
+      <c r="I22" s="4">
+        <v>0.06337301378887469</v>
+      </c>
+      <c r="J22" s="4">
+        <v>0.06514112262128603</v>
+      </c>
+      <c r="K22" s="4">
+        <v>89.7723704866562</v>
+      </c>
+      <c r="L22" s="4">
+        <v>93.48025296850801</v>
+      </c>
+      <c r="M22" s="5">
+        <v>104</v>
+      </c>
+      <c r="N22" s="5">
+        <v>99616.95075035095</v>
+      </c>
+      <c r="O22" s="4">
+        <v>25.28990879673799</v>
+      </c>
+      <c r="P22" s="5">
+        <v>3939</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="25" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="3">
+        <v>100</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4">
+        <v>0.06515784033802582</v>
+      </c>
+      <c r="I23" s="4">
+        <v>0.06515784033802582</v>
+      </c>
+      <c r="J23" s="4">
+        <v>0.06674250916375148</v>
+      </c>
+      <c r="K23" s="4">
+        <v>89.22782574568288</v>
+      </c>
+      <c r="L23" s="4">
+        <v>93.19469540526588</v>
+      </c>
+      <c r="M23" s="5">
+        <v>104</v>
+      </c>
+      <c r="N23" s="5">
+        <v>101589.7951126099</v>
+      </c>
+      <c r="O23" s="4">
+        <v>25.00979692580253</v>
+      </c>
+      <c r="P23" s="5">
+        <v>4062</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="25" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="3">
+        <v>100</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4">
+        <v>0.05521944141495191</v>
+      </c>
+      <c r="I24" s="4">
+        <v>0.05521944141495191</v>
+      </c>
+      <c r="J24" s="4">
+        <v>0.05777308623470101</v>
+      </c>
+      <c r="K24" s="4">
+        <v>89.70434327577185</v>
+      </c>
+      <c r="L24" s="4">
+        <v>93.45895715023229</v>
+      </c>
+      <c r="M24" s="5">
+        <v>104</v>
+      </c>
+      <c r="N24" s="5">
+        <v>571849.1594791412</v>
+      </c>
+      <c r="O24" s="4">
+        <v>143.2846804006869</v>
+      </c>
+      <c r="P24" s="5">
+        <v>3991</v>
       </c>
     </row>
   </sheetData>
@@ -1810,7 +3037,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1829,24 +3056,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
@@ -1869,25 +3096,25 @@
         <v>16</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="25" customHeight="1">
@@ -2071,13 +3298,13 @@
         <v>21</v>
       </c>
       <c r="B7" s="5">
-        <v>37</v>
+        <v>104</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
       </c>
       <c r="D7" s="5">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="E7" s="5">
         <v>0</v>
@@ -2086,7 +3313,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="5">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="H7" s="5">
         <v>0</v>
@@ -2115,13 +3342,13 @@
         <v>22</v>
       </c>
       <c r="B8" s="5">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
       </c>
       <c r="D8" s="5">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E8" s="5">
         <v>0</v>
@@ -2130,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="5">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5">
         <v>0</v>
@@ -2159,19 +3386,19 @@
         <v>23</v>
       </c>
       <c r="B9" s="5">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
       </c>
       <c r="D9" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5">
         <v>0</v>
       </c>
       <c r="F9" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9" s="5">
         <v>0</v>
@@ -2189,13 +3416,13 @@
         <v>0</v>
       </c>
       <c r="L9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" s="5">
         <v>0</v>
       </c>
       <c r="N9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="25" customHeight="1">
@@ -2203,13 +3430,13 @@
         <v>24</v>
       </c>
       <c r="B10" s="5">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
       </c>
       <c r="D10" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E10" s="5">
         <v>0</v>
@@ -2218,7 +3445,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H10" s="5">
         <v>0</v>
@@ -2247,13 +3474,13 @@
         <v>25</v>
       </c>
       <c r="B11" s="5">
-        <v>104</v>
+        <v>37</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
       </c>
       <c r="D11" s="5">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="E11" s="5">
         <v>0</v>
@@ -2262,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="5">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H11" s="5">
         <v>0</v>
@@ -2291,13 +3518,13 @@
         <v>26</v>
       </c>
       <c r="B12" s="5">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
       </c>
       <c r="D12" s="5">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E12" s="5">
         <v>0</v>
@@ -2306,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="5">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H12" s="5">
         <v>0</v>
@@ -2371,6 +3598,490 @@
         <v>0</v>
       </c>
       <c r="N13" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="25" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="5">
+        <v>104</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5">
+        <v>0</v>
+      </c>
+      <c r="K14" s="5">
+        <v>0</v>
+      </c>
+      <c r="L14" s="5">
+        <v>0</v>
+      </c>
+      <c r="M14" s="5">
+        <v>0</v>
+      </c>
+      <c r="N14" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5">
+        <v>104</v>
+      </c>
+      <c r="C15" s="5">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5">
+        <v>0</v>
+      </c>
+      <c r="K15" s="5">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5">
+        <v>0</v>
+      </c>
+      <c r="M15" s="5">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="25" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="5">
+        <v>104</v>
+      </c>
+      <c r="C16" s="5">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5">
+        <v>0</v>
+      </c>
+      <c r="J16" s="5">
+        <v>0</v>
+      </c>
+      <c r="K16" s="5">
+        <v>0</v>
+      </c>
+      <c r="L16" s="5">
+        <v>0</v>
+      </c>
+      <c r="M16" s="5">
+        <v>0</v>
+      </c>
+      <c r="N16" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="25" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="5">
+        <v>104</v>
+      </c>
+      <c r="C17" s="5">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5">
+        <v>0</v>
+      </c>
+      <c r="K17" s="5">
+        <v>0</v>
+      </c>
+      <c r="L17" s="5">
+        <v>0</v>
+      </c>
+      <c r="M17" s="5">
+        <v>0</v>
+      </c>
+      <c r="N17" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="25" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="5">
+        <v>104</v>
+      </c>
+      <c r="C18" s="5">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5">
+        <v>0</v>
+      </c>
+      <c r="I18" s="5">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5">
+        <v>0</v>
+      </c>
+      <c r="K18" s="5">
+        <v>0</v>
+      </c>
+      <c r="L18" s="5">
+        <v>0</v>
+      </c>
+      <c r="M18" s="5">
+        <v>0</v>
+      </c>
+      <c r="N18" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="25" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="5">
+        <v>104</v>
+      </c>
+      <c r="C19" s="5">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5">
+        <v>0</v>
+      </c>
+      <c r="J19" s="5">
+        <v>0</v>
+      </c>
+      <c r="K19" s="5">
+        <v>0</v>
+      </c>
+      <c r="L19" s="5">
+        <v>0</v>
+      </c>
+      <c r="M19" s="5">
+        <v>0</v>
+      </c>
+      <c r="N19" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="5">
+        <v>104</v>
+      </c>
+      <c r="C20" s="5">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5">
+        <v>0</v>
+      </c>
+      <c r="I20" s="5">
+        <v>0</v>
+      </c>
+      <c r="J20" s="5">
+        <v>0</v>
+      </c>
+      <c r="K20" s="5">
+        <v>0</v>
+      </c>
+      <c r="L20" s="5">
+        <v>0</v>
+      </c>
+      <c r="M20" s="5">
+        <v>0</v>
+      </c>
+      <c r="N20" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="25" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="5">
+        <v>26</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5">
+        <v>78</v>
+      </c>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5">
+        <v>78</v>
+      </c>
+      <c r="H21" s="5">
+        <v>0</v>
+      </c>
+      <c r="I21" s="5">
+        <v>0</v>
+      </c>
+      <c r="J21" s="5">
+        <v>0</v>
+      </c>
+      <c r="K21" s="5">
+        <v>0</v>
+      </c>
+      <c r="L21" s="5">
+        <v>0</v>
+      </c>
+      <c r="M21" s="5">
+        <v>0</v>
+      </c>
+      <c r="N21" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="25" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="5">
+        <v>104</v>
+      </c>
+      <c r="C22" s="5">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5">
+        <v>0</v>
+      </c>
+      <c r="I22" s="5">
+        <v>0</v>
+      </c>
+      <c r="J22" s="5">
+        <v>0</v>
+      </c>
+      <c r="K22" s="5">
+        <v>0</v>
+      </c>
+      <c r="L22" s="5">
+        <v>0</v>
+      </c>
+      <c r="M22" s="5">
+        <v>0</v>
+      </c>
+      <c r="N22" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="25" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="5">
+        <v>104</v>
+      </c>
+      <c r="C23" s="5">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5">
+        <v>0</v>
+      </c>
+      <c r="I23" s="5">
+        <v>0</v>
+      </c>
+      <c r="J23" s="5">
+        <v>0</v>
+      </c>
+      <c r="K23" s="5">
+        <v>0</v>
+      </c>
+      <c r="L23" s="5">
+        <v>0</v>
+      </c>
+      <c r="M23" s="5">
+        <v>0</v>
+      </c>
+      <c r="N23" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="25" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="5">
+        <v>104</v>
+      </c>
+      <c r="C24" s="5">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5">
+        <v>0</v>
+      </c>
+      <c r="H24" s="5">
+        <v>0</v>
+      </c>
+      <c r="I24" s="5">
+        <v>0</v>
+      </c>
+      <c r="J24" s="5">
+        <v>0</v>
+      </c>
+      <c r="K24" s="5">
+        <v>0</v>
+      </c>
+      <c r="L24" s="5">
+        <v>0</v>
+      </c>
+      <c r="M24" s="5">
+        <v>0</v>
+      </c>
+      <c r="N24" s="5">
         <v>0</v>
       </c>
     </row>
@@ -2389,7 +4100,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -2408,24 +4119,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
@@ -2448,25 +4159,25 @@
         <v>16</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="25" customHeight="1">
@@ -2738,19 +4449,19 @@
         <v>23</v>
       </c>
       <c r="B9" s="5">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
       </c>
       <c r="D9" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5">
         <v>0</v>
       </c>
       <c r="F9" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9" s="5">
         <v>0</v>
@@ -2768,13 +4479,13 @@
         <v>0</v>
       </c>
       <c r="L9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" s="5">
         <v>0</v>
       </c>
       <c r="N9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="25" customHeight="1">
@@ -2950,6 +4661,490 @@
         <v>0</v>
       </c>
       <c r="N13" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="25" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="5">
+        <v>104</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5">
+        <v>0</v>
+      </c>
+      <c r="K14" s="5">
+        <v>0</v>
+      </c>
+      <c r="L14" s="5">
+        <v>0</v>
+      </c>
+      <c r="M14" s="5">
+        <v>0</v>
+      </c>
+      <c r="N14" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5">
+        <v>104</v>
+      </c>
+      <c r="C15" s="5">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5">
+        <v>0</v>
+      </c>
+      <c r="K15" s="5">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5">
+        <v>0</v>
+      </c>
+      <c r="M15" s="5">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="25" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="5">
+        <v>104</v>
+      </c>
+      <c r="C16" s="5">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5">
+        <v>0</v>
+      </c>
+      <c r="J16" s="5">
+        <v>0</v>
+      </c>
+      <c r="K16" s="5">
+        <v>0</v>
+      </c>
+      <c r="L16" s="5">
+        <v>0</v>
+      </c>
+      <c r="M16" s="5">
+        <v>0</v>
+      </c>
+      <c r="N16" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="25" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="5">
+        <v>104</v>
+      </c>
+      <c r="C17" s="5">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5">
+        <v>0</v>
+      </c>
+      <c r="K17" s="5">
+        <v>0</v>
+      </c>
+      <c r="L17" s="5">
+        <v>0</v>
+      </c>
+      <c r="M17" s="5">
+        <v>0</v>
+      </c>
+      <c r="N17" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="25" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="5">
+        <v>104</v>
+      </c>
+      <c r="C18" s="5">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5">
+        <v>0</v>
+      </c>
+      <c r="I18" s="5">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5">
+        <v>0</v>
+      </c>
+      <c r="K18" s="5">
+        <v>0</v>
+      </c>
+      <c r="L18" s="5">
+        <v>0</v>
+      </c>
+      <c r="M18" s="5">
+        <v>0</v>
+      </c>
+      <c r="N18" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="25" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="5">
+        <v>104</v>
+      </c>
+      <c r="C19" s="5">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5">
+        <v>0</v>
+      </c>
+      <c r="J19" s="5">
+        <v>0</v>
+      </c>
+      <c r="K19" s="5">
+        <v>0</v>
+      </c>
+      <c r="L19" s="5">
+        <v>0</v>
+      </c>
+      <c r="M19" s="5">
+        <v>0</v>
+      </c>
+      <c r="N19" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="5">
+        <v>104</v>
+      </c>
+      <c r="C20" s="5">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5">
+        <v>0</v>
+      </c>
+      <c r="I20" s="5">
+        <v>0</v>
+      </c>
+      <c r="J20" s="5">
+        <v>0</v>
+      </c>
+      <c r="K20" s="5">
+        <v>0</v>
+      </c>
+      <c r="L20" s="5">
+        <v>0</v>
+      </c>
+      <c r="M20" s="5">
+        <v>0</v>
+      </c>
+      <c r="N20" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="25" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="5">
+        <v>104</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5">
+        <v>0</v>
+      </c>
+      <c r="I21" s="5">
+        <v>0</v>
+      </c>
+      <c r="J21" s="5">
+        <v>0</v>
+      </c>
+      <c r="K21" s="5">
+        <v>0</v>
+      </c>
+      <c r="L21" s="5">
+        <v>0</v>
+      </c>
+      <c r="M21" s="5">
+        <v>0</v>
+      </c>
+      <c r="N21" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="25" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="5">
+        <v>104</v>
+      </c>
+      <c r="C22" s="5">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5">
+        <v>0</v>
+      </c>
+      <c r="I22" s="5">
+        <v>0</v>
+      </c>
+      <c r="J22" s="5">
+        <v>0</v>
+      </c>
+      <c r="K22" s="5">
+        <v>0</v>
+      </c>
+      <c r="L22" s="5">
+        <v>0</v>
+      </c>
+      <c r="M22" s="5">
+        <v>0</v>
+      </c>
+      <c r="N22" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="25" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="5">
+        <v>104</v>
+      </c>
+      <c r="C23" s="5">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5">
+        <v>0</v>
+      </c>
+      <c r="I23" s="5">
+        <v>0</v>
+      </c>
+      <c r="J23" s="5">
+        <v>0</v>
+      </c>
+      <c r="K23" s="5">
+        <v>0</v>
+      </c>
+      <c r="L23" s="5">
+        <v>0</v>
+      </c>
+      <c r="M23" s="5">
+        <v>0</v>
+      </c>
+      <c r="N23" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="25" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="5">
+        <v>104</v>
+      </c>
+      <c r="C24" s="5">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5">
+        <v>0</v>
+      </c>
+      <c r="H24" s="5">
+        <v>0</v>
+      </c>
+      <c r="I24" s="5">
+        <v>0</v>
+      </c>
+      <c r="J24" s="5">
+        <v>0</v>
+      </c>
+      <c r="K24" s="5">
+        <v>0</v>
+      </c>
+      <c r="L24" s="5">
+        <v>0</v>
+      </c>
+      <c r="M24" s="5">
+        <v>0</v>
+      </c>
+      <c r="N24" s="5">
         <v>0</v>
       </c>
     </row>
@@ -2964,4 +5159,1073 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K34"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>104</v>
+      </c>
+      <c r="C2">
+        <v>104</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+      <c r="H2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" t="s">
+        <v>73</v>
+      </c>
+      <c r="K2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>104</v>
+      </c>
+      <c r="C3">
+        <v>104</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="H3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I3" t="s">
+        <v>72</v>
+      </c>
+      <c r="J3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4">
+        <v>104</v>
+      </c>
+      <c r="C4">
+        <v>104</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>100</v>
+      </c>
+      <c r="H4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4" t="s">
+        <v>73</v>
+      </c>
+      <c r="K4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5">
+        <v>104</v>
+      </c>
+      <c r="C5">
+        <v>104</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>100</v>
+      </c>
+      <c r="H5" t="s">
+        <v>71</v>
+      </c>
+      <c r="I5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J5" t="s">
+        <v>73</v>
+      </c>
+      <c r="K5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6">
+        <v>104</v>
+      </c>
+      <c r="C6">
+        <v>104</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="H6" t="s">
+        <v>71</v>
+      </c>
+      <c r="I6" t="s">
+        <v>72</v>
+      </c>
+      <c r="J6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7">
+        <v>104</v>
+      </c>
+      <c r="C7">
+        <v>104</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>100</v>
+      </c>
+      <c r="H7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J7" t="s">
+        <v>73</v>
+      </c>
+      <c r="K7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8">
+        <v>104</v>
+      </c>
+      <c r="C8">
+        <v>104</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>100</v>
+      </c>
+      <c r="H8" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" t="s">
+        <v>72</v>
+      </c>
+      <c r="J8" t="s">
+        <v>73</v>
+      </c>
+      <c r="K8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9">
+        <v>104</v>
+      </c>
+      <c r="C9">
+        <v>104</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" t="s">
+        <v>72</v>
+      </c>
+      <c r="J9" t="s">
+        <v>73</v>
+      </c>
+      <c r="K9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10">
+        <v>104</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>104</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" t="s">
+        <v>73</v>
+      </c>
+      <c r="K10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11">
+        <v>104</v>
+      </c>
+      <c r="C11">
+        <v>104</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>100</v>
+      </c>
+      <c r="H11" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" t="s">
+        <v>72</v>
+      </c>
+      <c r="J11" t="s">
+        <v>73</v>
+      </c>
+      <c r="K11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12">
+        <v>104</v>
+      </c>
+      <c r="C12">
+        <v>104</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>100</v>
+      </c>
+      <c r="H12" t="s">
+        <v>71</v>
+      </c>
+      <c r="I12" t="s">
+        <v>72</v>
+      </c>
+      <c r="J12" t="s">
+        <v>73</v>
+      </c>
+      <c r="K12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13">
+        <v>104</v>
+      </c>
+      <c r="C13">
+        <v>104</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>100</v>
+      </c>
+      <c r="H13" t="s">
+        <v>71</v>
+      </c>
+      <c r="I13" t="s">
+        <v>72</v>
+      </c>
+      <c r="J13" t="s">
+        <v>73</v>
+      </c>
+      <c r="K13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14">
+        <v>104</v>
+      </c>
+      <c r="C14">
+        <v>104</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>100</v>
+      </c>
+      <c r="H14" t="s">
+        <v>71</v>
+      </c>
+      <c r="I14" t="s">
+        <v>72</v>
+      </c>
+      <c r="J14" t="s">
+        <v>73</v>
+      </c>
+      <c r="K14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15">
+        <v>104</v>
+      </c>
+      <c r="C15">
+        <v>104</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>100</v>
+      </c>
+      <c r="H15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J15" t="s">
+        <v>73</v>
+      </c>
+      <c r="K15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16">
+        <v>104</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>104</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
+        <v>70</v>
+      </c>
+      <c r="H16" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" t="s">
+        <v>72</v>
+      </c>
+      <c r="J16" t="s">
+        <v>73</v>
+      </c>
+      <c r="K16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17">
+        <v>104</v>
+      </c>
+      <c r="C17">
+        <v>104</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>100</v>
+      </c>
+      <c r="H17" t="s">
+        <v>71</v>
+      </c>
+      <c r="I17" t="s">
+        <v>72</v>
+      </c>
+      <c r="J17" t="s">
+        <v>73</v>
+      </c>
+      <c r="K17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18">
+        <v>104</v>
+      </c>
+      <c r="C18">
+        <v>104</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>100</v>
+      </c>
+      <c r="H18" t="s">
+        <v>71</v>
+      </c>
+      <c r="I18" t="s">
+        <v>72</v>
+      </c>
+      <c r="J18" t="s">
+        <v>73</v>
+      </c>
+      <c r="K18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19">
+        <v>104</v>
+      </c>
+      <c r="C19">
+        <v>104</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>100</v>
+      </c>
+      <c r="H19" t="s">
+        <v>71</v>
+      </c>
+      <c r="I19" t="s">
+        <v>72</v>
+      </c>
+      <c r="J19" t="s">
+        <v>73</v>
+      </c>
+      <c r="K19" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20">
+        <v>104</v>
+      </c>
+      <c r="C20">
+        <v>104</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>100</v>
+      </c>
+      <c r="H20" t="s">
+        <v>71</v>
+      </c>
+      <c r="I20" t="s">
+        <v>72</v>
+      </c>
+      <c r="J20" t="s">
+        <v>73</v>
+      </c>
+      <c r="K20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21">
+        <v>104</v>
+      </c>
+      <c r="C21">
+        <v>104</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>100</v>
+      </c>
+      <c r="H21" t="s">
+        <v>71</v>
+      </c>
+      <c r="I21" t="s">
+        <v>72</v>
+      </c>
+      <c r="J21" t="s">
+        <v>73</v>
+      </c>
+      <c r="K21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22">
+        <v>104</v>
+      </c>
+      <c r="C22">
+        <v>104</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>100</v>
+      </c>
+      <c r="H22" t="s">
+        <v>71</v>
+      </c>
+      <c r="I22" t="s">
+        <v>72</v>
+      </c>
+      <c r="J22" t="s">
+        <v>73</v>
+      </c>
+      <c r="K22" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23">
+        <v>104</v>
+      </c>
+      <c r="C23">
+        <v>104</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>100</v>
+      </c>
+      <c r="H23" t="s">
+        <v>71</v>
+      </c>
+      <c r="I23" t="s">
+        <v>72</v>
+      </c>
+      <c r="J23" t="s">
+        <v>73</v>
+      </c>
+      <c r="K23" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24">
+        <v>104</v>
+      </c>
+      <c r="C24">
+        <v>104</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>100</v>
+      </c>
+      <c r="H24" t="s">
+        <v>71</v>
+      </c>
+      <c r="I24" t="s">
+        <v>72</v>
+      </c>
+      <c r="J24" t="s">
+        <v>73</v>
+      </c>
+      <c r="K24" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25">
+        <v>104</v>
+      </c>
+      <c r="C25">
+        <v>104</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>100</v>
+      </c>
+      <c r="H25" t="s">
+        <v>71</v>
+      </c>
+      <c r="I25" t="s">
+        <v>72</v>
+      </c>
+      <c r="J25" t="s">
+        <v>73</v>
+      </c>
+      <c r="K25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26">
+        <v>104</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>104</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H26" t="s">
+        <v>71</v>
+      </c>
+      <c r="I26" t="s">
+        <v>72</v>
+      </c>
+      <c r="J26" t="s">
+        <v>73</v>
+      </c>
+      <c r="K26" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27">
+        <v>104</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>104</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="s">
+        <v>70</v>
+      </c>
+      <c r="H27" t="s">
+        <v>71</v>
+      </c>
+      <c r="I27" t="s">
+        <v>72</v>
+      </c>
+      <c r="J27" t="s">
+        <v>73</v>
+      </c>
+      <c r="K27" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" t="s">
+        <v>65</v>
+      </c>
+      <c r="B28">
+        <v>104</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>104</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" t="s">
+        <v>70</v>
+      </c>
+      <c r="H28" t="s">
+        <v>71</v>
+      </c>
+      <c r="I28" t="s">
+        <v>72</v>
+      </c>
+      <c r="J28" t="s">
+        <v>73</v>
+      </c>
+      <c r="K28" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
+      <c r="A29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29">
+        <v>104</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>104</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29" t="s">
+        <v>70</v>
+      </c>
+      <c r="H29" t="s">
+        <v>71</v>
+      </c>
+      <c r="I29" t="s">
+        <v>72</v>
+      </c>
+      <c r="J29" t="s">
+        <v>73</v>
+      </c>
+      <c r="K29" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30">
+        <v>104</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>104</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30" t="s">
+        <v>70</v>
+      </c>
+      <c r="H30" t="s">
+        <v>71</v>
+      </c>
+      <c r="I30" t="s">
+        <v>72</v>
+      </c>
+      <c r="J30" t="s">
+        <v>73</v>
+      </c>
+      <c r="K30" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
+      <c r="A31" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31">
+        <v>104</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>104</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31" t="s">
+        <v>70</v>
+      </c>
+      <c r="H31" t="s">
+        <v>71</v>
+      </c>
+      <c r="I31" t="s">
+        <v>72</v>
+      </c>
+      <c r="J31" t="s">
+        <v>73</v>
+      </c>
+      <c r="K31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
+      <c r="A32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32">
+        <v>104</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>104</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32" t="s">
+        <v>70</v>
+      </c>
+      <c r="H32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J32" t="s">
+        <v>73</v>
+      </c>
+      <c r="K32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>